<commit_message>
qbo to qbo africa
</commit_message>
<xml_diff>
--- a/server/data/Adjustmentnote/modifiedAdjustmentnote.xlsx
+++ b/server/data/Adjustmentnote/modifiedAdjustmentnote.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ _€"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -397,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -466,34 +467,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>101</v>
+        <v>2442</v>
       </c>
       <c r="B2" t="str">
-        <v>Aiman N (deleted)</v>
-      </c>
-      <c r="C2">
-        <v>45879</v>
+        <v>IUA Business Solutions</v>
+      </c>
+      <c r="C2" t="str">
+        <v>22/03/2024</v>
       </c>
       <c r="D2" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>25/03/2024</v>
       </c>
       <c r="F2" t="str">
         <v>Sales</v>
       </c>
       <c r="G2" t="str">
-        <v>Created by QB Online to adjust balance for deletion</v>
+        <v>For return of 32 x 2m, Cat 6 flyleads</v>
       </c>
       <c r="H2" t="str">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="I2">
-        <v>3442.36</v>
+        <v>35</v>
       </c>
       <c r="J2">
-        <v>3442.36</v>
+        <v>1120</v>
       </c>
       <c r="K2" t="str">
         <v>Out Of Scope</v>
@@ -531,34 +532,34 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>102</v>
+        <v>2538</v>
       </c>
       <c r="B3" t="str">
-        <v>Alex H (deleted)</v>
-      </c>
-      <c r="C3">
-        <v>45879</v>
+        <v>Geckosoft</v>
+      </c>
+      <c r="C3" t="str">
+        <v>07/05/2024</v>
       </c>
       <c r="D3" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>07/05/2024</v>
       </c>
       <c r="F3" t="str">
         <v>Sales</v>
       </c>
       <c r="G3" t="str">
-        <v>Created by QB Online to adjust balance for deletion</v>
+        <v>Credit refund for invoice 2523</v>
       </c>
       <c r="H3" t="str">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>767.82</v>
+        <v>909.57</v>
       </c>
       <c r="J3">
-        <v>767.82</v>
+        <v>909.57</v>
       </c>
       <c r="K3" t="str">
         <v>Out Of Scope</v>
@@ -596,34 +597,34 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>7691</v>
+        <v>2597</v>
       </c>
       <c r="B4" t="str">
-        <v>David Golos (deleted)</v>
-      </c>
-      <c r="C4">
-        <v>45565</v>
+        <v>Netelligent Consulting CC</v>
+      </c>
+      <c r="C4" t="str">
+        <v>03/06/2024</v>
       </c>
       <c r="D4" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>03/06/2024</v>
       </c>
       <c r="F4" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Credit Note for Tag Reader invoiced (2567) on the 22nd May 2024 in error</v>
       </c>
       <c r="H4" t="str">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>306.88</v>
+        <v>2125</v>
       </c>
       <c r="J4">
-        <v>306.88</v>
+        <v>2125</v>
       </c>
       <c r="K4" t="str">
         <v>Out Of Scope</v>
@@ -661,34 +662,34 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>7692</v>
+        <v>2607/2608/2609</v>
       </c>
       <c r="B5" t="str">
-        <v>Rick De Tommaso (deleted)</v>
-      </c>
-      <c r="C5">
-        <v>45565</v>
+        <v>PSi IT Services</v>
+      </c>
+      <c r="C5" t="str">
+        <v>05/06/2024</v>
       </c>
       <c r="D5" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>05/06/2024</v>
       </c>
       <c r="F5" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G5" t="str">
-        <v>Unpaid invoice</v>
+        <v>Credit Note For invoices 2607,2608 &amp; 2609 issued 5th June 2024</v>
       </c>
       <c r="H5" t="str">
         <v>1</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>109424.5</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>109424.5</v>
       </c>
       <c r="K5" t="str">
         <v>Out Of Scope</v>
@@ -726,34 +727,34 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>7693</v>
+        <v>2629</v>
       </c>
       <c r="B6" t="str">
-        <v>Rick De Tommaso (deleted)</v>
-      </c>
-      <c r="C6">
-        <v>45565</v>
+        <v>Reflex Solutions Pty Ltd</v>
+      </c>
+      <c r="C6" t="str">
+        <v>11/06/2024</v>
       </c>
       <c r="D6" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>11/06/2024</v>
       </c>
       <c r="F6" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>Credit Note for labour as per invoice 2624 dd 10 June 2024- Volpes The Crescent</v>
       </c>
       <c r="H6" t="str">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>281.88</v>
+        <v>2000</v>
       </c>
       <c r="J6">
-        <v>281.88</v>
+        <v>2000</v>
       </c>
       <c r="K6" t="str">
         <v>Out Of Scope</v>
@@ -791,34 +792,34 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>7694</v>
+        <v>2661</v>
       </c>
       <c r="B7" t="str">
-        <v>Rick De Tommaso (deleted)</v>
-      </c>
-      <c r="C7">
-        <v>45565</v>
+        <v>American Consulate General Durban</v>
+      </c>
+      <c r="C7" t="str">
+        <v>02/07/2024</v>
       </c>
       <c r="D7" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>02/07/2024</v>
       </c>
       <c r="F7" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>CN Issued for Invoice 2661 - New invoice 2666 issued with correct costings dd 7 July 2024</v>
       </c>
       <c r="H7" t="str">
         <v>1</v>
       </c>
       <c r="I7">
-        <v>546.29</v>
+        <v>1672</v>
       </c>
       <c r="J7">
-        <v>546.29</v>
+        <v>1672</v>
       </c>
       <c r="K7" t="str">
         <v>Out Of Scope</v>
@@ -856,34 +857,34 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>7695</v>
+        <v>2682</v>
       </c>
       <c r="B8" t="str">
-        <v>Stewart Watson (deleted)</v>
-      </c>
-      <c r="C8">
-        <v>45565</v>
+        <v>American Consulate General Durban</v>
+      </c>
+      <c r="C8" t="str">
+        <v>09/07/2024</v>
       </c>
       <c r="D8" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>09/07/2024</v>
       </c>
       <c r="F8" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>Credit note issues for invoice 2610 dd 5 June 2024- CGR Phone &amp; wi fi license- New invoice  issued  No. 2681 dd 9 July 2024 with correct costing and PO No.</v>
       </c>
       <c r="H8" t="str">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>279.77</v>
+        <v>1210</v>
       </c>
       <c r="J8">
-        <v>279.77</v>
+        <v>1210</v>
       </c>
       <c r="K8" t="str">
         <v>Out Of Scope</v>
@@ -921,34 +922,34 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7696</v>
+        <v>2685</v>
       </c>
       <c r="B9" t="str">
-        <v>Maree Barron (deleted)</v>
-      </c>
-      <c r="C9">
-        <v>45565</v>
+        <v>Tuatara Technology (Pty) Ltd</v>
+      </c>
+      <c r="C9" t="str">
+        <v>05/07/2024</v>
       </c>
       <c r="D9" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>05/07/2024</v>
       </c>
       <c r="F9" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>REFUND FOR LTE ROUTER AS PER Q10265</v>
       </c>
       <c r="H9" t="str">
         <v>1</v>
       </c>
       <c r="I9">
-        <v>861.5</v>
+        <v>1500</v>
       </c>
       <c r="J9">
-        <v>861.5</v>
+        <v>1500</v>
       </c>
       <c r="K9" t="str">
         <v>Out Of Scope</v>
@@ -986,13 +987,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>7697</v>
+        <v>2685</v>
       </c>
       <c r="B10" t="str">
-        <v>Adam Przezdziecki (deleted)</v>
-      </c>
-      <c r="C10">
-        <v>45565</v>
+        <v>Tuatara Technology (Pty) Ltd</v>
+      </c>
+      <c r="C10" t="str">
+        <v>05/07/2024</v>
       </c>
       <c r="D10" t="str">
         <v>TaxExcluded</v>
@@ -1001,7 +1002,7 @@
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Bad Debt</v>
+        <v/>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -1010,10 +1011,10 @@
         <v>1</v>
       </c>
       <c r="I10">
-        <v>1959.76</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>1959.76</v>
+        <v>0</v>
       </c>
       <c r="K10" t="str">
         <v>Out Of Scope</v>
@@ -1051,34 +1052,34 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>7698</v>
+        <v>2798</v>
       </c>
       <c r="B11" t="str">
-        <v>Carolyn Song (deleted)</v>
-      </c>
-      <c r="C11">
-        <v>45565</v>
+        <v>Boltfix</v>
+      </c>
+      <c r="C11" t="str">
+        <v>05/09/2024</v>
       </c>
       <c r="D11" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>04/09/2024</v>
       </c>
       <c r="F11" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>Over charged on SLA Warehouse</v>
       </c>
       <c r="H11" t="str">
         <v>1</v>
       </c>
       <c r="I11">
-        <v>936.21</v>
+        <v>149.57</v>
       </c>
       <c r="J11">
-        <v>936.21</v>
+        <v>149.57</v>
       </c>
       <c r="K11" t="str">
         <v>Out Of Scope</v>
@@ -1116,34 +1117,34 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>7699</v>
+        <v>2837</v>
       </c>
       <c r="B12" t="str">
-        <v>David Golos (deleted)</v>
-      </c>
-      <c r="C12">
-        <v>45565</v>
+        <v>Colab IT Solutions Pty Ltd</v>
+      </c>
+      <c r="C12" t="str">
+        <v>30/09/2024</v>
       </c>
       <c r="D12" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>30/09/2024</v>
       </c>
       <c r="F12" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G12" t="str">
-        <v/>
+        <v>Extra Points charged on the incorrect PO. PowaFix- Cato Ridge</v>
       </c>
       <c r="H12" t="str">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>45</v>
+        <v>2805</v>
       </c>
       <c r="J12">
-        <v>45</v>
+        <v>2805</v>
       </c>
       <c r="K12" t="str">
         <v>Out Of Scope</v>
@@ -1181,13 +1182,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>7700</v>
+        <v>2929</v>
       </c>
       <c r="B13" t="str">
-        <v>Mark Kinsman (deleted)</v>
-      </c>
-      <c r="C13">
-        <v>45565</v>
+        <v>Starrate IT</v>
+      </c>
+      <c r="C13" t="str">
+        <v>22/11/2024</v>
       </c>
       <c r="D13" t="str">
         <v>TaxExcluded</v>
@@ -1196,19 +1197,19 @@
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>PO9144</v>
       </c>
       <c r="H13" t="str">
         <v>1</v>
       </c>
       <c r="I13">
-        <v>1697.44</v>
+        <v>775</v>
       </c>
       <c r="J13">
-        <v>1697.44</v>
+        <v>775</v>
       </c>
       <c r="K13" t="str">
         <v>Out Of Scope</v>
@@ -1246,34 +1247,34 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>7701</v>
+        <v>3035</v>
       </c>
       <c r="B14" t="str">
-        <v>Maxim Gunner (deleted)</v>
-      </c>
-      <c r="C14">
-        <v>45565</v>
+        <v>Beast Leather</v>
+      </c>
+      <c r="C14" t="str">
+        <v>03/02/2025</v>
       </c>
       <c r="D14" t="str">
         <v>TaxExcluded</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>04/02/2025</v>
       </c>
       <c r="F14" t="str">
-        <v>Bad Debt</v>
+        <v>Sales</v>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>W/O unable to get the funds</v>
       </c>
       <c r="H14" t="str">
         <v>1</v>
       </c>
       <c r="I14">
-        <v>4109.46</v>
+        <v>4115</v>
       </c>
       <c r="J14">
-        <v>4109.46</v>
+        <v>4115</v>
       </c>
       <c r="K14" t="str">
         <v>Out Of Scope</v>
@@ -1306,12 +1307,402 @@
         <v/>
       </c>
       <c r="U14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>3036</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Cubix Solutions (PTY) LTD</v>
+      </c>
+      <c r="C15" t="str">
+        <v>04/02/2025</v>
+      </c>
+      <c r="D15" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E15" t="str">
+        <v>04/02/2025</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="G15" t="str">
+        <v>W/O 0.75</v>
+      </c>
+      <c r="H15" t="str">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0.65</v>
+      </c>
+      <c r="J15">
+        <v>0.65</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>3076</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Pro Hydraulics (Pty) Ltd</v>
+      </c>
+      <c r="C16" t="str">
+        <v>07/04/2025</v>
+      </c>
+      <c r="D16" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E16" t="str">
+        <v>07/04/2025</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Over charged day labour</v>
+      </c>
+      <c r="H16" t="str">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>4000</v>
+      </c>
+      <c r="J16">
+        <v>4000</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>3233</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Rowena Scott</v>
+      </c>
+      <c r="C17" t="str">
+        <v>02/06/2025</v>
+      </c>
+      <c r="D17" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E17" t="str">
+        <v>04/06/2025</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Write Off</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Write off- old balance</v>
+      </c>
+      <c r="H17" t="str">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>10</v>
+      </c>
+      <c r="J17">
+        <v>10</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>3233</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Rowena Scott</v>
+      </c>
+      <c r="C18" t="str">
+        <v>02/06/2025</v>
+      </c>
+      <c r="D18" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>3264</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Starrate IT</v>
+      </c>
+      <c r="C19" t="str">
+        <v>24/06/2025</v>
+      </c>
+      <c r="D19" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="G19" t="str">
+        <v>PO9577</v>
+      </c>
+      <c r="H19" t="str">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>25830</v>
+      </c>
+      <c r="J19">
+        <v>25830</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>3271</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PSi IT Services</v>
+      </c>
+      <c r="C20" t="str">
+        <v>26/06/2025</v>
+      </c>
+      <c r="D20" t="str">
+        <v>TaxExcluded</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="G20" t="str">
+        <v>PO1469</v>
+      </c>
+      <c r="H20" t="str">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>48385</v>
+      </c>
+      <c r="J20">
+        <v>48385</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Out Of Scope</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>